<commit_message>
Fix: FRACAS writing to project-specific file - Kayseri yazılı Belgrad'ın dosyasına değil, Kayseri/Fracas_KAYSERI.xlsx'e yaz
</commit_message>
<xml_diff>
--- a/data/kayseri/service_status.xlsx
+++ b/data/kayseri/service_status.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,22 +471,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Servis Dışı</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Traction_Converter</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Tahrik Konvertörü Sis.  Kontaktör</t>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-03-02 09:40:37</t>
+          <t>2026-03-02 14:24:55</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -518,7 +513,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-03-02 09:34:06</t>
+          <t>2026-03-02 14:24:55</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -540,15 +535,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>İşletme Kaynaklı Servis Dışı</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-03-02 09:40:46</t>
+          <t>2026-03-02 14:24:55</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -580,7 +577,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-03-02 09:34:06</t>
+          <t>2026-03-02 14:24:55</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -612,7 +609,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-03-02 09:34:06</t>
+          <t>2026-03-02 14:24:56</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -666,17 +663,23 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Servis</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Toplu servise alındı</t>
-        </is>
-      </c>
+          <t>Servis Dışı</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Wiper_System</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Silecek Mekanızması</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-03-02 09:34:06</t>
+          <t>2026-03-02 14:27:17</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -808,6 +811,710 @@
         </is>
       </c>
       <c r="H12" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>3872</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:02</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>3873</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:02</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>3874</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:02</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>3875</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:02</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>3876</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:02</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>3877</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:02</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>3878</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:02</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>3879</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:02</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>3880</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:03</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>3881</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:03</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>3882</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:03</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>3872</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:19</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>3873</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:19</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>3874</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:19</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>3875</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:20</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>3876</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:20</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>3877</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:20</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>3878</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:20</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>3879</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:20</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>3880</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:20</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>3881</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:20</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>3882</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:26:21</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
         <is>
           <t>admin</t>
         </is>

</xml_diff>